<commit_message>
conversie de date, operatii cu stringuri, block-uri decizionale
</commit_message>
<xml_diff>
--- a/Programare I/Prezenta Programare.xlsx
+++ b/Programare I/Prezenta Programare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Geoinformatica_Promotia_2026_2029\Programare I\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC00097-447B-40EB-BB3F-F9452398CE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5ACCE27-EE4F-494C-B9AD-D264B14048C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Prenume Nume</t>
   </si>
@@ -81,9 +81,6 @@
     <t>Mihai Sebastian Barb</t>
   </si>
   <si>
-    <t>Marian Catalin Pacurar</t>
-  </si>
-  <si>
     <t>Claudia Pop</t>
   </si>
   <si>
@@ -108,10 +105,16 @@
     <t>Antonia Petrasca</t>
   </si>
   <si>
-    <t>Klara Gratiela Virag</t>
-  </si>
-  <si>
     <t>Iulia Fekete Novak</t>
+  </si>
+  <si>
+    <t>Catalin Pacurar</t>
+  </si>
+  <si>
+    <t>Gratiela Virag</t>
+  </si>
+  <si>
+    <t>Alexandru Grama</t>
   </si>
 </sst>
 </file>
@@ -715,12 +718,12 @@
     </row>
     <row r="3" spans="2:18">
       <c r="B3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="5">
-        <v>1</v>
-      </c>
-      <c r="D3" s="6"/>
+        <v>29</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="6">
+        <v>1</v>
+      </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -741,35 +744,52 @@
     </row>
     <row r="4" spans="2:18">
       <c r="B4" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C4" s="9">
         <v>1</v>
       </c>
+      <c r="D4" s="15">
+        <v>1</v>
+      </c>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
       <c r="P4" s="10"/>
       <c r="Q4" s="8">
         <f>SUM(C4:P4)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R4" s="10"/>
     </row>
     <row r="5" spans="2:18">
       <c r="B5" s="4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C5" s="9">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
         <v>1</v>
       </c>
       <c r="P5" s="10"/>
       <c r="Q5" s="8">
         <f>SUM(C5:P5)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5" s="10"/>
     </row>
     <row r="6" spans="2:18">
       <c r="B6" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C6" s="9">
         <v>1</v>
@@ -783,15 +803,18 @@
     </row>
     <row r="7" spans="2:18">
       <c r="B7" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C7" s="9">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3">
         <v>1</v>
       </c>
       <c r="P7" s="10"/>
       <c r="Q7" s="8">
         <f>SUM(C7:P7)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" s="10"/>
     </row>
@@ -802,44 +825,53 @@
       <c r="C8" s="9">
         <v>1</v>
       </c>
+      <c r="D8" s="3">
+        <v>1</v>
+      </c>
       <c r="P8" s="10"/>
       <c r="Q8" s="8">
         <f>SUM(C8:P8)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R8" s="10"/>
     </row>
     <row r="9" spans="2:18">
       <c r="B9" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C9" s="9">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3">
         <v>1</v>
       </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="8">
         <f>SUM(C9:P9)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="10"/>
     </row>
     <row r="10" spans="2:18">
       <c r="B10" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="9">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3">
         <v>1</v>
       </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
         <f>SUM(C10:P10)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="10"/>
     </row>
     <row r="11" spans="2:18">
       <c r="B11" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C11" s="9">
         <v>1</v>
@@ -853,7 +885,7 @@
     </row>
     <row r="12" spans="2:18">
       <c r="B12" s="4" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C12" s="9">
         <v>1</v>
@@ -867,23 +899,11 @@
     </row>
     <row r="13" spans="2:18">
       <c r="B13" s="4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C13" s="9">
         <v>1</v>
       </c>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
-      <c r="N13" s="15"/>
-      <c r="O13" s="15"/>
       <c r="P13" s="10"/>
       <c r="Q13" s="8">
         <f>SUM(C13:P13)</f>
@@ -893,25 +913,35 @@
     </row>
     <row r="14" spans="2:18">
       <c r="B14" s="4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C14" s="9">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3">
         <v>1</v>
       </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="8">
         <f>SUM(C14:P14)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" s="10"/>
     </row>
     <row r="15" spans="2:18">
-      <c r="B15" s="4"/>
-      <c r="C15" s="9"/>
+      <c r="B15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="9">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1</v>
+      </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="8">
-        <f t="shared" ref="Q3:Q22" si="0">SUM(C15:P15)</f>
-        <v>0</v>
+        <f>SUM(C15:P15)</f>
+        <v>2</v>
       </c>
       <c r="R15" s="10"/>
     </row>
@@ -920,7 +950,7 @@
       <c r="C16" s="9"/>
       <c r="P16" s="10"/>
       <c r="Q16" s="8">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="Q15:Q22" si="0">SUM(C16:P16)</f>
         <v>0</v>
       </c>
       <c r="R16" s="10"/>
@@ -1298,8 +1328,8 @@
       <c r="R52" s="14"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:R14">
-    <sortCondition ref="B3:B14"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:R15">
+    <sortCondition ref="B3:B15"/>
   </sortState>
   <conditionalFormatting sqref="Q3:Q52">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>

<commit_message>
Enum, Struct, Maximul dintre 3 numere
</commit_message>
<xml_diff>
--- a/Programare I/Prezenta Programare.xlsx
+++ b/Programare I/Prezenta Programare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Geoinformatica_Promotia_2026_2029\Programare I\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5ACCE27-EE4F-494C-B9AD-D264B14048C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BCA5621-1AC1-41AE-9113-FDBEBAA1A5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Prenume Nume</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Nota</t>
   </si>
   <si>
-    <t>Mihai Sebastian Barb</t>
-  </si>
-  <si>
     <t>Claudia Pop</t>
   </si>
   <si>
@@ -115,6 +112,21 @@
   </si>
   <si>
     <t>Alexandru Grama</t>
+  </si>
+  <si>
+    <t>Sebastian Barb</t>
+  </si>
+  <si>
+    <t>Lorena Mester</t>
+  </si>
+  <si>
+    <t>Mark Maier</t>
+  </si>
+  <si>
+    <t>Darius Zbarcea</t>
+  </si>
+  <si>
+    <t>Eduard Pop</t>
   </si>
 </sst>
 </file>
@@ -314,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -356,9 +368,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -718,13 +727,15 @@
     </row>
     <row r="3" spans="2:18">
       <c r="B3" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="6">
         <v>1</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="6">
+        <v>1</v>
+      </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -738,58 +749,53 @@
       <c r="P3" s="7"/>
       <c r="Q3" s="8">
         <f>SUM(C3:P3)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R3" s="7"/>
     </row>
     <row r="4" spans="2:18">
       <c r="B4" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" s="9">
         <v>1</v>
       </c>
-      <c r="D4" s="15">
-        <v>1</v>
-      </c>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
+      <c r="D4" s="3">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
       <c r="P4" s="10"/>
       <c r="Q4" s="8">
         <f>SUM(C4:P4)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R4" s="10"/>
     </row>
     <row r="5" spans="2:18">
       <c r="B5" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" s="9">
         <v>1</v>
       </c>
       <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3">
         <v>1</v>
       </c>
       <c r="P5" s="10"/>
       <c r="Q5" s="8">
         <f>SUM(C5:P5)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R5" s="10"/>
     </row>
     <row r="6" spans="2:18">
       <c r="B6" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="9">
         <v>1</v>
@@ -803,77 +809,85 @@
     </row>
     <row r="7" spans="2:18">
       <c r="B7" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="9">
         <v>1</v>
       </c>
       <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3">
         <v>1</v>
       </c>
       <c r="P7" s="10"/>
       <c r="Q7" s="8">
         <f>SUM(C7:P7)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7" s="10"/>
     </row>
     <row r="8" spans="2:18">
       <c r="B8" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="9">
         <v>1</v>
       </c>
       <c r="D8" s="3">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3">
         <v>1</v>
       </c>
       <c r="P8" s="10"/>
       <c r="Q8" s="8">
         <f>SUM(C8:P8)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R8" s="10"/>
     </row>
     <row r="9" spans="2:18">
       <c r="B9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="9">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3">
+        <v>32</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="E9" s="3">
         <v>1</v>
       </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="8">
         <f>SUM(C9:P9)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="10"/>
     </row>
     <row r="10" spans="2:18">
       <c r="B10" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C10" s="9">
         <v>1</v>
       </c>
       <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3">
         <v>1</v>
       </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
         <f>SUM(C10:P10)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="10"/>
     </row>
     <row r="11" spans="2:18">
       <c r="B11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="9">
+        <v>33</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="E11" s="3">
         <v>1</v>
       </c>
       <c r="P11" s="10"/>
@@ -885,103 +899,136 @@
     </row>
     <row r="12" spans="2:18">
       <c r="B12" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C12" s="9">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
         <v>1</v>
       </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="8">
         <f>SUM(C12:P12)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R12" s="10"/>
     </row>
     <row r="13" spans="2:18">
       <c r="B13" s="4" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C13" s="9">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3">
         <v>1</v>
       </c>
       <c r="P13" s="10"/>
       <c r="Q13" s="8">
         <f>SUM(C13:P13)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R13" s="10"/>
     </row>
     <row r="14" spans="2:18">
       <c r="B14" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C14" s="9">
-        <v>1</v>
-      </c>
-      <c r="D14" s="3">
         <v>1</v>
       </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="8">
         <f>SUM(C14:P14)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="10"/>
     </row>
     <row r="15" spans="2:18">
       <c r="B15" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="9">
-        <v>1</v>
-      </c>
-      <c r="D15" s="3">
+        <v>30</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="E15" s="3">
         <v>1</v>
       </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="8">
         <f>SUM(C15:P15)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R15" s="10"/>
     </row>
     <row r="16" spans="2:18">
-      <c r="B16" s="4"/>
-      <c r="C16" s="9"/>
+      <c r="B16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="9">
+        <v>1</v>
+      </c>
       <c r="P16" s="10"/>
       <c r="Q16" s="8">
-        <f t="shared" ref="Q15:Q22" si="0">SUM(C16:P16)</f>
-        <v>0</v>
+        <f>SUM(C16:P16)</f>
+        <v>1</v>
       </c>
       <c r="R16" s="10"/>
     </row>
     <row r="17" spans="2:18">
-      <c r="B17" s="4"/>
+      <c r="B17" s="4" t="s">
+        <v>31</v>
+      </c>
       <c r="C17" s="9"/>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
       <c r="P17" s="10"/>
       <c r="Q17" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(C17:P17)</f>
+        <v>1</v>
       </c>
       <c r="R17" s="10"/>
     </row>
     <row r="18" spans="2:18">
-      <c r="B18" s="4"/>
-      <c r="C18" s="9"/>
+      <c r="B18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="9">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3">
+        <v>1</v>
+      </c>
       <c r="P18" s="10"/>
       <c r="Q18" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(C18:P18)</f>
+        <v>3</v>
       </c>
       <c r="R18" s="10"/>
     </row>
     <row r="19" spans="2:18">
-      <c r="B19" s="4"/>
-      <c r="C19" s="9"/>
+      <c r="B19" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="9">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1</v>
+      </c>
       <c r="P19" s="10"/>
       <c r="Q19" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(C19:P19)</f>
+        <v>3</v>
       </c>
       <c r="R19" s="10"/>
     </row>
@@ -990,7 +1037,7 @@
       <c r="C20" s="9"/>
       <c r="P20" s="10"/>
       <c r="Q20" s="8">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="Q16:Q22" si="0">SUM(C20:P20)</f>
         <v>0</v>
       </c>
       <c r="R20" s="10"/>
@@ -1328,8 +1375,8 @@
       <c r="R52" s="14"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:R15">
-    <sortCondition ref="B3:B15"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:R19">
+    <sortCondition ref="B3:B19"/>
   </sortState>
   <conditionalFormatting sqref="Q3:Q52">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>